<commit_message>
Daily attendance processing - 2026-06-21 13:37:05 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7">
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8">
@@ -964,7 +964,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>43.0%</t>
+          <t>43.3%</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>80.1%</t>
         </is>
       </c>
     </row>
@@ -1318,22 +1318,22 @@
         <v>40</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>18</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>32.5%</t>
+          <t>35.0%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>83.8%</t>
+          <t>84.9%</t>
         </is>
       </c>
     </row>
@@ -2614,45 +2614,49 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>A2A1</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>RHEUMATOLOGY</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>21/06/2026</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>37/37</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -9641,7 +9645,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11437,7 +11441,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13018,7 +13022,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13065,7 +13069,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14814,7 +14818,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -14861,7 +14865,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-23 20:09:31 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7">
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -964,7 +964,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>47.0%</t>
+          <t>47.7%</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>80.7%</t>
+          <t>80.4%</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1806,22 @@
         <v>40</v>
       </c>
       <c r="O21" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q21" s="4" t="n">
         <v>16</v>
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
-          <t>52.5%</t>
+          <t>55.0%</t>
         </is>
       </c>
       <c r="S21" s="4" t="inlineStr">
         <is>
-          <t>86.3%</t>
+          <t>86.6%</t>
         </is>
       </c>
     </row>
@@ -1884,22 +1884,22 @@
         <v>40</v>
       </c>
       <c r="O22" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>16</v>
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>52.5%</t>
+          <t>55.0%</t>
         </is>
       </c>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>75.8%</t>
         </is>
       </c>
     </row>
@@ -9677,7 +9677,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11477,7 +11477,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -12420,45 +12420,49 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B256" s="2" t="inlineStr">
+      <c r="A256" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B256" s="5" t="inlineStr">
         <is>
           <t>A2D1</t>
         </is>
       </c>
-      <c r="C256" s="2" t="inlineStr">
+      <c r="C256" s="5" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D256" s="2" t="inlineStr">
+      <c r="D256" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E256" s="2" t="inlineStr">
+      <c r="E256" s="5" t="inlineStr">
         <is>
           <t>23/06/2026</t>
         </is>
       </c>
-      <c r="F256" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G256" s="2" t="inlineStr"/>
-      <c r="H256" s="2" t="inlineStr">
-        <is>
-          <t>0/34</t>
-        </is>
-      </c>
-      <c r="I256" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F256" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G256" s="5" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H256" s="5" t="inlineStr">
+        <is>
+          <t>32/34</t>
+        </is>
+      </c>
+      <c r="I256" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -14224,45 +14228,49 @@
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B296" s="2" t="inlineStr">
+      <c r="A296" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B296" s="5" t="inlineStr">
         <is>
           <t>A2D2</t>
         </is>
       </c>
-      <c r="C296" s="2" t="inlineStr">
+      <c r="C296" s="5" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D296" s="2" t="inlineStr">
+      <c r="D296" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E296" s="2" t="inlineStr">
+      <c r="E296" s="5" t="inlineStr">
         <is>
           <t>23/06/2026</t>
         </is>
       </c>
-      <c r="F296" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G296" s="2" t="inlineStr"/>
-      <c r="H296" s="2" t="inlineStr">
-        <is>
-          <t>0/40</t>
-        </is>
-      </c>
-      <c r="I296" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F296" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G296" s="5" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H296" s="5" t="inlineStr">
+        <is>
+          <t>7/40</t>
+        </is>
+      </c>
+      <c r="I296" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-23 21:43:34 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9677,7 +9677,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11477,7 +11477,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13113,7 +13113,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14921,7 +14921,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-24 00:08:02 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9677,7 +9677,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11477,7 +11477,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13066,7 +13066,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13113,7 +13113,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -14921,7 +14921,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-25 16:34:33 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13094,7 +13094,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14906,7 +14906,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -14953,7 +14953,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-26 21:19:02 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13094,7 +13094,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14906,7 +14906,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -14953,7 +14953,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-28 20:06:43 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13142,7 +13142,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13189,7 +13189,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14958,7 +14958,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15005,7 +15005,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-28 21:11:30 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9737,7 +9737,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11549,7 +11549,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13142,7 +13142,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13189,7 +13189,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -14958,7 +14958,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15005,7 +15005,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-29 16:57:39 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9757,7 +9757,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11573,7 +11573,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13213,7 +13213,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-30 13:34:16 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13233,7 +13233,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-06-30 16:16:04 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13233,7 +13233,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-01 16:18:53 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13206,7 +13206,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13253,7 +13253,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15034,7 +15034,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15081,7 +15081,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-04 22:09:02 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9805,7 +9805,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11625,7 +11625,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13277,7 +13277,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15109,7 +15109,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-09 14:18:02 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9869,7 +9869,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11697,7 +11697,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13302,7 +13302,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15150,7 +15150,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15197,7 +15197,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-09 19:04:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13302,7 +13302,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15150,7 +15150,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15197,7 +15197,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-10 06:54:06 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9869,7 +9869,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11697,7 +11697,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15197,7 +15197,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-10 20:37:49 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9869,7 +9869,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11697,7 +11697,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-11 00:05:02 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13349,7 +13349,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15197,7 +15197,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-11 07:38:00 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>222</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7">
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
@@ -964,7 +964,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>69.2%</t>
+          <t>70.4%</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>78.1%</t>
+          <t>77.6%</t>
         </is>
       </c>
     </row>
@@ -1318,22 +1318,22 @@
         <v>40</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="P15" s="4" t="n">
         <v>8</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>67.5%</t>
+          <t>70.0%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>79.1%</t>
+          <t>77.4%</t>
         </is>
       </c>
     </row>
@@ -1400,22 +1400,22 @@
         <v>41</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>11</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>61.0%</t>
+          <t>63.4%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>79.5%</t>
+          <t>78.5%</t>
         </is>
       </c>
     </row>
@@ -1481,10 +1481,10 @@
         <v>29</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
@@ -1563,10 +1563,10 @@
         <v>28</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
@@ -1642,22 +1642,22 @@
         <v>40</v>
       </c>
       <c r="O19" s="4" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P19" s="4" t="n">
         <v>5</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R19" s="4" t="inlineStr">
         <is>
-          <t>75.0%</t>
+          <t>77.5%</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>77.4%</t>
+          <t>77.2%</t>
         </is>
       </c>
     </row>
@@ -1724,22 +1724,22 @@
         <v>40</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>10</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>62.5%</t>
+          <t>65.0%</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>80.4%</t>
+          <t>79.3%</t>
         </is>
       </c>
     </row>
@@ -1809,10 +1809,10 @@
         <v>26</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
@@ -1891,10 +1891,10 @@
         <v>32</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
@@ -2349,45 +2349,49 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>A2A1</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>NEUROLOGY</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G31" s="9" t="inlineStr"/>
-      <c r="H31" s="9" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I31" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>12/37</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -4208,45 +4212,49 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="9" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B72" s="9" t="inlineStr">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
         <is>
           <t>A2A2</t>
         </is>
       </c>
-      <c r="C72" s="9" t="inlineStr">
+      <c r="C72" s="5" t="inlineStr">
         <is>
           <t>NEUROLOGY</t>
         </is>
       </c>
-      <c r="D72" s="9" t="inlineStr">
+      <c r="D72" s="5" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E72" s="9" t="inlineStr">
+      <c r="E72" s="5" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="F72" s="9" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G72" s="9" t="inlineStr"/>
-      <c r="H72" s="9" t="inlineStr">
-        <is>
-          <t>0/35</t>
-        </is>
-      </c>
-      <c r="I72" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>18/35</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -4932,45 +4940,45 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="9" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B88" s="9" t="inlineStr">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>A2B1</t>
         </is>
       </c>
-      <c r="C88" s="9" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>ENDOCRINOLOGY</t>
         </is>
       </c>
-      <c r="D88" s="9" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E88" s="9" t="inlineStr">
+      <c r="E88" s="2" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="F88" s="9" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G88" s="9" t="inlineStr"/>
-      <c r="H88" s="9" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr">
         <is>
           <t>0/37</t>
         </is>
       </c>
-      <c r="I88" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -6768,45 +6776,45 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="9" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B128" s="9" t="inlineStr">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>A2B2</t>
         </is>
       </c>
-      <c r="C128" s="9" t="inlineStr">
+      <c r="C128" s="2" t="inlineStr">
         <is>
           <t>ENDOCRINOLOGY</t>
         </is>
       </c>
-      <c r="D128" s="9" t="inlineStr">
+      <c r="D128" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E128" s="9" t="inlineStr">
+      <c r="E128" s="2" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="F128" s="9" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G128" s="9" t="inlineStr"/>
-      <c r="H128" s="9" t="inlineStr">
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr"/>
+      <c r="H128" s="2" t="inlineStr">
         <is>
           <t>0/36</t>
         </is>
       </c>
-      <c r="I128" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -9066,45 +9074,49 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="9" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B178" s="9" t="inlineStr">
+      <c r="A178" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B178" s="5" t="inlineStr">
         <is>
           <t>A2C1</t>
         </is>
       </c>
-      <c r="C178" s="9" t="inlineStr">
+      <c r="C178" s="5" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D178" s="9" t="inlineStr">
+      <c r="D178" s="5" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E178" s="9" t="inlineStr">
+      <c r="E178" s="5" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="F178" s="9" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G178" s="9" t="inlineStr"/>
-      <c r="H178" s="9" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I178" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F178" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G178" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H178" s="5" t="inlineStr">
+        <is>
+          <t>26/37</t>
+        </is>
+      </c>
+      <c r="I178" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -10894,45 +10906,49 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="9" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B218" s="9" t="inlineStr">
+      <c r="A218" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B218" s="5" t="inlineStr">
         <is>
           <t>A2C2</t>
         </is>
       </c>
-      <c r="C218" s="9" t="inlineStr">
+      <c r="C218" s="5" t="inlineStr">
         <is>
           <t>GASTROENTEROLOGY</t>
         </is>
       </c>
-      <c r="D218" s="9" t="inlineStr">
+      <c r="D218" s="5" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E218" s="9" t="inlineStr">
+      <c r="E218" s="5" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="F218" s="9" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G218" s="9" t="inlineStr"/>
-      <c r="H218" s="9" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I218" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F218" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G218" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H218" s="5" t="inlineStr">
+        <is>
+          <t>19/37</t>
+        </is>
+      </c>
+      <c r="I218" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -12961,45 +12977,45 @@
       </c>
     </row>
     <row r="263">
-      <c r="A263" s="9" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B263" s="9" t="inlineStr">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
         <is>
           <t>A2D1</t>
         </is>
       </c>
-      <c r="C263" s="9" t="inlineStr">
+      <c r="C263" s="2" t="inlineStr">
         <is>
           <t>NEPHROLOGY</t>
         </is>
       </c>
-      <c r="D263" s="9" t="inlineStr">
+      <c r="D263" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E263" s="9" t="inlineStr">
+      <c r="E263" s="2" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="F263" s="9" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G263" s="9" t="inlineStr"/>
-      <c r="H263" s="9" t="inlineStr">
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr"/>
+      <c r="H263" s="2" t="inlineStr">
         <is>
           <t>0/34</t>
         </is>
       </c>
-      <c r="I263" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I263" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>
@@ -15490,45 +15506,45 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="9" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B318" s="9" t="inlineStr">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B318" s="2" t="inlineStr">
         <is>
           <t>A2D2</t>
         </is>
       </c>
-      <c r="C318" s="9" t="inlineStr">
+      <c r="C318" s="2" t="inlineStr">
         <is>
           <t>RHEUMATOLOGY</t>
         </is>
       </c>
-      <c r="D318" s="9" t="inlineStr">
+      <c r="D318" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E318" s="9" t="inlineStr">
+      <c r="E318" s="2" t="inlineStr">
         <is>
           <t>11/07/2026</t>
         </is>
       </c>
-      <c r="F318" s="9" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G318" s="9" t="inlineStr"/>
-      <c r="H318" s="9" t="inlineStr">
+      <c r="F318" s="2" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G318" s="2" t="inlineStr"/>
+      <c r="H318" s="2" t="inlineStr">
         <is>
           <t>0/40</t>
         </is>
       </c>
-      <c r="I318" s="9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I318" s="2" t="inlineStr">
+        <is>
+          <t>Not Recorded</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-11 12:04:00 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>77.9%</t>
+          <t>78.1%</t>
         </is>
       </c>
     </row>
@@ -1739,7 +1739,7 @@
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>79.3%</t>
+          <t>80.9%</t>
         </is>
       </c>
     </row>
@@ -9889,7 +9889,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -10951,7 +10951,7 @@
       </c>
       <c r="H218" s="5" t="inlineStr">
         <is>
-          <t>19/37</t>
+          <t>34/37</t>
         </is>
       </c>
       <c r="I218" s="5" t="inlineStr">
@@ -11721,7 +11721,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13330,7 +13330,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15225,7 +15225,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-11 14:48:59 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9114,7 +9114,7 @@
       </c>
       <c r="G178" s="5" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H178" s="5" t="inlineStr">
@@ -10946,7 +10946,7 @@
       </c>
       <c r="G218" s="5" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H218" s="5" t="inlineStr">
@@ -13330,7 +13330,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15225,7 +15225,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-12 09:39:29 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7">
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8">
@@ -964,7 +964,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>71.7%</t>
+          <t>72.3%</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>78.1%</t>
+          <t>78.2%</t>
         </is>
       </c>
     </row>
@@ -1318,22 +1318,22 @@
         <v>40</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>70.0%</t>
+          <t>72.5%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>78.5%</t>
         </is>
       </c>
     </row>
@@ -1400,22 +1400,22 @@
         <v>41</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>3</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>63.4%</t>
+          <t>65.9%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>79.5%</t>
+          <t>79.8%</t>
         </is>
       </c>
     </row>
@@ -2396,45 +2396,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>A2A1</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>NEUROLOGY</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>12/07/2026</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>28/37</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -4259,45 +4263,49 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>A2A2</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>NEUROLOGY</t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="E73" s="5" t="inlineStr">
         <is>
           <t>12/07/2026</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr"/>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>0/35</t>
-        </is>
-      </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>31/35</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -9889,7 +9897,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11721,7 +11729,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13377,7 +13385,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15225,7 +15233,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-12 14:53:04 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13358,7 +13358,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13405,7 +13405,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15206,7 +15206,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-12 16:09:50 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13358,7 +13358,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13405,7 +13405,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15206,7 +15206,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-12 19:18:45 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9909,7 +9909,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11745,7 +11745,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13405,7 +13405,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-13 17:07:15 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9937,7 +9937,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11777,7 +11777,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13394,7 +13394,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13441,7 +13441,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15242,7 +15242,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15289,7 +15289,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-14 14:36:02 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9957,7 +9957,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11801,7 +11801,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13465,7 +13465,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15313,7 +15313,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-15 09:41:00 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7">
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8">
@@ -961,7 +961,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>78.8%</t>
+          <t>79.4%</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>77.9%</t>
         </is>
       </c>
     </row>
@@ -1315,17 +1315,17 @@
         <v>40</v>
       </c>
       <c r="O15" s="4" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>77.5%</t>
+          <t>80.0%</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
@@ -1397,22 +1397,22 @@
         <v>41</v>
       </c>
       <c r="O16" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>70.7%</t>
+          <t>73.2%</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>78.7%</t>
+          <t>79.4%</t>
         </is>
       </c>
     </row>
@@ -2581,45 +2581,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>A2A1</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>PHYSICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>15/07/2026</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>0/37</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>28/37</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -4456,45 +4460,49 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>Year 5</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
         <is>
           <t>A2A2</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C77" s="5" t="inlineStr">
         <is>
           <t>PHYSICAL MEDICINE</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D77" s="5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E77" s="5" t="inlineStr">
         <is>
           <t>15/07/2026</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>09:00:00</t>
-        </is>
-      </c>
-      <c r="G77" s="2" t="inlineStr"/>
-      <c r="H77" s="2" t="inlineStr">
-        <is>
-          <t>0/35</t>
-        </is>
-      </c>
-      <c r="I77" s="2" t="inlineStr">
-        <is>
-          <t>Not Recorded</t>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>2026/2027</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>35/35</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>Recorded</t>
         </is>
       </c>
     </row>
@@ -9954,7 +9962,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11798,7 +11806,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13462,7 +13470,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15310,7 +15318,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-15 14:58:31 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9966,7 +9966,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15330,7 +15330,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-15 17:58:41 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9966,7 +9966,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-15 19:17:25 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13482,7 +13482,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15330,7 +15330,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-17 06:46:14 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13443,7 +13443,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13490,7 +13490,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15291,7 +15291,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15338,7 +15338,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-17 09:17:51 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13443,7 +13443,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13490,7 +13490,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15291,7 +15291,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15338,7 +15338,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-17 17:46:56 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-18 10:08:05 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-18 12:06:28 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-19 17:08:10 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2026/2027, 2025/2026</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-19 18:05:54 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-19 22:37:52 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-19 23:41:30 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-21 16:33:17 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-22 20:05:44 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-23 15:20:26 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-24 04:23:51 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-24 19:09:34 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-28 23:14:07 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-29 14:50:13 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-07-30 18:05:07 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-02 08:23:44 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-02 11:49:56 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-02 18:11:48 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-02 19:50:54 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-02 23:00:49 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2025/2026, 2027/2028</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-03 17:56:01 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2026/2027, 2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-05 02:09:46 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-05 13:05:56 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-05 15:20:40 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-06 00:05:31 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-07 00:03:13 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028</t>
+          <t>2027/2028, 2025/2026</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2027/2028, 2025/2026, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-07 14:18:33 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-07 16:32:03 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2026/2027, 2027/2028, 2025/2026</t>
+          <t>2027/2028, 2026/2027, 2025/2026</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-08 12:02:31 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-08 18:04:52 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-08 23:08:15 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-09 11:11:10 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 160715@med.asu.edu.eg</t>
+          <t>160715@med.asu.edu.eg, 2025/2026</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-09 12:03:15 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2026/2027, 2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-10 11:14:36 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13451,7 +13451,7 @@
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H270" s="5" t="inlineStr">
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15299,7 +15299,7 @@
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026</t>
+          <t>2025/2026, 2027/2028</t>
         </is>
       </c>
       <c r="H310" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2027/2028, 2025/2026, 2026/2027</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-11 08:18:57 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-11 15:02:41 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-12 03:43:42 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2026/2027, 2027/2028</t>
+          <t>2025/2026, 2027/2028, 2026/2027</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-12 13:05:20 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -13498,7 +13498,7 @@
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H271" s="5" t="inlineStr">
@@ -15346,7 +15346,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>2025/2026, 2027/2028, 2026/2027</t>
+          <t>2025/2026, 2026/2027, 2027/2028</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Daily attendance processing - 2026-08-12 22:44:29 UTC
</commit_message>
<xml_diff>
--- a/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
+++ b/attendance_reports/Y5_B2526_General_&_Special_Internal_2_A2_session_analysis.xlsx
@@ -9974,7 +9974,7 @@
       </c>
       <c r="G195" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H195" s="5" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>160715@med.asu.edu.eg, 2025/2026</t>
+          <t>2025/2026, 160715@med.asu.edu.eg</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">

</xml_diff>